<commit_message>
Update dvs.xlsx markup: 12000-45000 range per user spec
</commit_message>
<xml_diff>
--- a/dvs.xlsx
+++ b/dvs.xlsx
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="AH5" t="n">
-        <v>336000</v>
+        <v>364000</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="AH6" t="n">
-        <v>193000</v>
+        <v>209000</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="AH7" t="n">
-        <v>193000</v>
+        <v>209000</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="AH8" t="n">
-        <v>193000</v>
+        <v>209000</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="AH9" t="n">
-        <v>325500</v>
+        <v>353000</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
@@ -2196,7 +2196,7 @@
         </is>
       </c>
       <c r="AH10" t="n">
-        <v>111000</v>
+        <v>120500</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="AH11" t="n">
-        <v>108000</v>
+        <v>117500</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
@@ -2378,7 +2378,7 @@
         </is>
       </c>
       <c r="AH12" t="n">
-        <v>108000</v>
+        <v>117500</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="AH13" t="n">
-        <v>108000</v>
+        <v>117500</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="AH14" t="n">
-        <v>95500</v>
+        <v>104000</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="AH15" t="n">
-        <v>141500</v>
+        <v>154000</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
@@ -2742,7 +2742,7 @@
         </is>
       </c>
       <c r="AH16" t="n">
-        <v>141500</v>
+        <v>154000</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="AH17" t="n">
-        <v>172500</v>
+        <v>187000</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
@@ -2924,7 +2924,7 @@
         </is>
       </c>
       <c r="AH18" t="n">
-        <v>121500</v>
+        <v>131500</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="AH19" t="n">
-        <v>116000</v>
+        <v>126000</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="AH20" t="n">
-        <v>105000</v>
+        <v>114000</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="AH21" t="n">
-        <v>103000</v>
+        <v>112000</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
@@ -3288,7 +3288,7 @@
         </is>
       </c>
       <c r="AH22" t="n">
-        <v>101000</v>
+        <v>109500</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="AH23" t="n">
-        <v>101000</v>
+        <v>109500</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="AH24" t="n">
-        <v>101000</v>
+        <v>109500</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
@@ -3561,7 +3561,7 @@
         </is>
       </c>
       <c r="AH25" t="n">
-        <v>49500</v>
+        <v>54500</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="AH26" t="n">
-        <v>213000</v>
+        <v>231000</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
@@ -3743,7 +3743,7 @@
         </is>
       </c>
       <c r="AH27" t="n">
-        <v>60000</v>
+        <v>65500</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
@@ -3834,7 +3834,7 @@
         </is>
       </c>
       <c r="AH28" t="n">
-        <v>60000</v>
+        <v>65500</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="AH29" t="n">
-        <v>58000</v>
+        <v>63000</v>
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
@@ -4016,7 +4016,7 @@
         </is>
       </c>
       <c r="AH30" t="n">
-        <v>53000</v>
+        <v>57500</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="AH31" t="n">
-        <v>187500</v>
+        <v>203500</v>
       </c>
       <c r="AJ31" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
         </is>
       </c>
       <c r="AH32" t="n">
-        <v>177500</v>
+        <v>192500</v>
       </c>
       <c r="AJ32" t="inlineStr">
         <is>
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="AH33" t="n">
-        <v>111000</v>
+        <v>120500</v>
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="AH34" t="n">
-        <v>172500</v>
+        <v>187000</v>
       </c>
       <c r="AJ34" t="inlineStr">
         <is>
@@ -4471,7 +4471,7 @@
         </is>
       </c>
       <c r="AH35" t="n">
-        <v>126500</v>
+        <v>137500</v>
       </c>
       <c r="AJ35" t="inlineStr">
         <is>
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="AH36" t="n">
-        <v>85500</v>
+        <v>93000</v>
       </c>
       <c r="AJ36" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
         </is>
       </c>
       <c r="AH37" t="n">
-        <v>44500</v>
+        <v>49000</v>
       </c>
       <c r="AJ37" t="inlineStr">
         <is>
@@ -4744,7 +4744,7 @@
         </is>
       </c>
       <c r="AH38" t="n">
-        <v>29500</v>
+        <v>32000</v>
       </c>
       <c r="AJ38" t="inlineStr">
         <is>
@@ -4835,7 +4835,7 @@
         </is>
       </c>
       <c r="AH39" t="n">
-        <v>27500</v>
+        <v>30000</v>
       </c>
       <c r="AJ39" t="inlineStr">
         <is>
@@ -4926,7 +4926,7 @@
         </is>
       </c>
       <c r="AH40" t="n">
-        <v>315500</v>
+        <v>342000</v>
       </c>
       <c r="AJ40" t="inlineStr">
         <is>
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="AH41" t="n">
-        <v>208000</v>
+        <v>225500</v>
       </c>
       <c r="AJ41" t="inlineStr">
         <is>
@@ -5108,7 +5108,7 @@
         </is>
       </c>
       <c r="AH42" t="n">
-        <v>203000</v>
+        <v>220000</v>
       </c>
       <c r="AJ42" t="inlineStr">
         <is>
@@ -5199,7 +5199,7 @@
         </is>
       </c>
       <c r="AH43" t="n">
-        <v>187500</v>
+        <v>203500</v>
       </c>
       <c r="AJ43" t="inlineStr">
         <is>
@@ -5290,7 +5290,7 @@
         </is>
       </c>
       <c r="AH44" t="n">
-        <v>121500</v>
+        <v>131500</v>
       </c>
       <c r="AJ44" t="inlineStr">
         <is>
@@ -5381,7 +5381,7 @@
         </is>
       </c>
       <c r="AH45" t="n">
-        <v>121500</v>
+        <v>131500</v>
       </c>
       <c r="AJ45" t="inlineStr">
         <is>
@@ -5472,7 +5472,7 @@
         </is>
       </c>
       <c r="AH46" t="n">
-        <v>99000</v>
+        <v>107500</v>
       </c>
       <c r="AJ46" t="inlineStr">
         <is>
@@ -5563,7 +5563,7 @@
         </is>
       </c>
       <c r="AH47" t="n">
-        <v>90500</v>
+        <v>98500</v>
       </c>
       <c r="AJ47" t="inlineStr">
         <is>
@@ -5654,7 +5654,7 @@
         </is>
       </c>
       <c r="AH48" t="n">
-        <v>182500</v>
+        <v>198000</v>
       </c>
       <c r="AJ48" t="inlineStr">
         <is>
@@ -5745,7 +5745,7 @@
         </is>
       </c>
       <c r="AH49" t="n">
-        <v>162000</v>
+        <v>176000</v>
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="AH50" t="n">
-        <v>141500</v>
+        <v>154000</v>
       </c>
       <c r="AJ50" t="inlineStr">
         <is>
@@ -5927,7 +5927,7 @@
         </is>
       </c>
       <c r="AH51" t="n">
-        <v>131500</v>
+        <v>143000</v>
       </c>
       <c r="AJ51" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
         </is>
       </c>
       <c r="AH52" t="n">
-        <v>198000</v>
+        <v>214500</v>
       </c>
       <c r="AJ52" t="inlineStr">
         <is>
@@ -6109,7 +6109,7 @@
         </is>
       </c>
       <c r="AH53" t="n">
-        <v>223500</v>
+        <v>242500</v>
       </c>
       <c r="AJ53" t="inlineStr">
         <is>
@@ -6200,7 +6200,7 @@
         </is>
       </c>
       <c r="AH54" t="n">
-        <v>346000</v>
+        <v>375000</v>
       </c>
       <c r="AJ54" t="inlineStr">
         <is>
@@ -6291,7 +6291,7 @@
         </is>
       </c>
       <c r="AH55" t="n">
-        <v>126500</v>
+        <v>137500</v>
       </c>
       <c r="AJ55" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
       <c r="AH56" t="n">
-        <v>49500</v>
+        <v>54500</v>
       </c>
       <c r="AJ56" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
         </is>
       </c>
       <c r="AH57" t="n">
-        <v>131500</v>
+        <v>143000</v>
       </c>
       <c r="AJ57" t="inlineStr">
         <is>
@@ -6564,7 +6564,7 @@
         </is>
       </c>
       <c r="AH58" t="n">
-        <v>116000</v>
+        <v>126000</v>
       </c>
       <c r="AJ58" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="AH59" t="n">
-        <v>106000</v>
+        <v>115000</v>
       </c>
       <c r="AJ59" t="inlineStr">
         <is>
@@ -6746,7 +6746,7 @@
         </is>
       </c>
       <c r="AH60" t="n">
-        <v>65000</v>
+        <v>71000</v>
       </c>
       <c r="AJ60" t="inlineStr">
         <is>
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="AH61" t="n">
-        <v>65000</v>
+        <v>71000</v>
       </c>
       <c r="AJ61" t="inlineStr">
         <is>
@@ -6928,7 +6928,7 @@
         </is>
       </c>
       <c r="AH62" t="n">
-        <v>90500</v>
+        <v>98500</v>
       </c>
       <c r="AJ62" t="inlineStr">
         <is>
@@ -7019,7 +7019,7 @@
         </is>
       </c>
       <c r="AH63" t="n">
-        <v>80500</v>
+        <v>87500</v>
       </c>
       <c r="AJ63" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="AH64" t="n">
-        <v>76500</v>
+        <v>83000</v>
       </c>
       <c r="AJ64" t="inlineStr">
         <is>
@@ -7201,7 +7201,7 @@
         </is>
       </c>
       <c r="AH65" t="n">
-        <v>60000</v>
+        <v>65500</v>
       </c>
       <c r="AJ65" t="inlineStr">
         <is>
@@ -7292,7 +7292,7 @@
         </is>
       </c>
       <c r="AH66" t="n">
-        <v>57000</v>
+        <v>62000</v>
       </c>
       <c r="AJ66" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="AH67" t="n">
-        <v>52000</v>
+        <v>56500</v>
       </c>
       <c r="AJ67" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="AH68" t="n">
-        <v>49500</v>
+        <v>54500</v>
       </c>
       <c r="AJ68" t="inlineStr">
         <is>
@@ -7565,7 +7565,7 @@
         </is>
       </c>
       <c r="AH69" t="n">
-        <v>32500</v>
+        <v>35500</v>
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
@@ -7656,7 +7656,7 @@
         </is>
       </c>
       <c r="AH70" t="n">
-        <v>131500</v>
+        <v>143000</v>
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
@@ -7747,7 +7747,7 @@
         </is>
       </c>
       <c r="AH71" t="n">
-        <v>116000</v>
+        <v>126000</v>
       </c>
       <c r="AJ71" t="inlineStr">
         <is>
@@ -7838,7 +7838,7 @@
         </is>
       </c>
       <c r="AH72" t="n">
-        <v>60000</v>
+        <v>65500</v>
       </c>
       <c r="AJ72" t="inlineStr">
         <is>
@@ -7929,7 +7929,7 @@
         </is>
       </c>
       <c r="AH73" t="n">
-        <v>95500</v>
+        <v>104000</v>
       </c>
       <c r="AJ73" t="inlineStr">
         <is>
@@ -8020,7 +8020,7 @@
         </is>
       </c>
       <c r="AH74" t="n">
-        <v>131500</v>
+        <v>143000</v>
       </c>
       <c r="AJ74" t="inlineStr">
         <is>
@@ -8111,7 +8111,7 @@
         </is>
       </c>
       <c r="AH75" t="n">
-        <v>131500</v>
+        <v>143000</v>
       </c>
       <c r="AJ75" t="inlineStr">
         <is>
@@ -8202,7 +8202,7 @@
         </is>
       </c>
       <c r="AH76" t="n">
-        <v>80500</v>
+        <v>87500</v>
       </c>
       <c r="AJ76" t="inlineStr">
         <is>
@@ -8293,7 +8293,7 @@
         </is>
       </c>
       <c r="AH77" t="n">
-        <v>95500</v>
+        <v>104000</v>
       </c>
       <c r="AJ77" t="inlineStr">
         <is>
@@ -8384,7 +8384,7 @@
         </is>
       </c>
       <c r="AH78" t="n">
-        <v>68000</v>
+        <v>74000</v>
       </c>
       <c r="AJ78" t="inlineStr">
         <is>
@@ -8475,7 +8475,7 @@
         </is>
       </c>
       <c r="AH79" t="n">
-        <v>141500</v>
+        <v>154000</v>
       </c>
       <c r="AJ79" t="inlineStr">
         <is>
@@ -8566,7 +8566,7 @@
         </is>
       </c>
       <c r="AH80" t="n">
-        <v>187500</v>
+        <v>203500</v>
       </c>
       <c r="AJ80" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
         </is>
       </c>
       <c r="AH81" t="n">
-        <v>187500</v>
+        <v>203500</v>
       </c>
       <c r="AJ81" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
         </is>
       </c>
       <c r="AH82" t="n">
-        <v>180500</v>
+        <v>196000</v>
       </c>
       <c r="AJ82" t="inlineStr">
         <is>
@@ -8839,7 +8839,7 @@
         </is>
       </c>
       <c r="AH83" t="n">
-        <v>141500</v>
+        <v>154000</v>
       </c>
       <c r="AJ83" t="inlineStr">
         <is>
@@ -8930,7 +8930,7 @@
         </is>
       </c>
       <c r="AH84" t="n">
-        <v>121500</v>
+        <v>131500</v>
       </c>
       <c r="AJ84" t="inlineStr">
         <is>
@@ -9021,7 +9021,7 @@
         </is>
       </c>
       <c r="AH85" t="n">
-        <v>95500</v>
+        <v>104000</v>
       </c>
       <c r="AJ85" t="inlineStr">
         <is>
@@ -9112,7 +9112,7 @@
         </is>
       </c>
       <c r="AH86" t="n">
-        <v>90500</v>
+        <v>98500</v>
       </c>
       <c r="AJ86" t="inlineStr">
         <is>
@@ -9203,7 +9203,7 @@
         </is>
       </c>
       <c r="AH87" t="n">
-        <v>90500</v>
+        <v>98500</v>
       </c>
       <c r="AJ87" t="inlineStr">
         <is>
@@ -9294,7 +9294,7 @@
         </is>
       </c>
       <c r="AH88" t="n">
-        <v>101000</v>
+        <v>109500</v>
       </c>
       <c r="AJ88" t="inlineStr">
         <is>
@@ -9385,7 +9385,7 @@
         </is>
       </c>
       <c r="AH89" t="n">
-        <v>67000</v>
+        <v>73000</v>
       </c>
       <c r="AJ89" t="inlineStr">
         <is>

</xml_diff>